<commit_message>
Fix Report Filtering, Add BADLAR Chart, Automatize API Data retrieval and Updates Github Workflow
</commit_message>
<xml_diff>
--- a/seriesAPI_BCRA_Digest.xlsx
+++ b/seriesAPI_BCRA_Digest.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1541"/>
+  <dimension ref="A1:H1542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10869,7 +10869,7 @@
         <v>3922697</v>
       </c>
       <c r="D496" t="n">
-        <v>108.48</v>
+        <v>108.29</v>
       </c>
       <c r="E496" t="n">
         <v>34.1875</v>
@@ -10891,7 +10891,7 @@
         <v>3851298</v>
       </c>
       <c r="D497" t="n">
-        <v>108.61</v>
+        <v>108.48</v>
       </c>
       <c r="E497" t="n">
         <v>34.25</v>
@@ -10913,7 +10913,7 @@
         <v>3950424</v>
       </c>
       <c r="D498" t="n">
-        <v>108.63</v>
+        <v>108.61</v>
       </c>
       <c r="E498" t="n">
         <v>34.25</v>
@@ -10935,7 +10935,7 @@
         <v>4326335</v>
       </c>
       <c r="D499" t="n">
-        <v>108.72</v>
+        <v>108.63</v>
       </c>
       <c r="E499" t="n">
         <v>34.1875</v>
@@ -10957,7 +10957,7 @@
         <v>3761928</v>
       </c>
       <c r="D500" t="n">
-        <v>108.86</v>
+        <v>108.72</v>
       </c>
       <c r="E500" t="n">
         <v>37.375</v>
@@ -10979,7 +10979,7 @@
         <v>3780254</v>
       </c>
       <c r="D501" t="n">
-        <v>108.96</v>
+        <v>108.86</v>
       </c>
       <c r="E501" t="n">
         <v>37.625</v>
@@ -11001,7 +11001,7 @@
         <v>3569643</v>
       </c>
       <c r="D502" t="n">
-        <v>108.97</v>
+        <v>108.96</v>
       </c>
       <c r="E502" t="n">
         <v>37.375</v>
@@ -11023,7 +11023,7 @@
         <v>3602002</v>
       </c>
       <c r="D503" t="n">
-        <v>109.05</v>
+        <v>108.97</v>
       </c>
       <c r="E503" t="n">
         <v>37.4375</v>
@@ -11045,7 +11045,7 @@
         <v>3521623</v>
       </c>
       <c r="D504" t="n">
-        <v>109.11</v>
+        <v>109.05</v>
       </c>
       <c r="E504" t="n">
         <v>37.4375</v>
@@ -11067,7 +11067,7 @@
         <v>3644760</v>
       </c>
       <c r="D505" t="n">
-        <v>109.21</v>
+        <v>109.11</v>
       </c>
       <c r="E505" t="n">
         <v>37.625</v>
@@ -11089,7 +11089,7 @@
         <v>3772372</v>
       </c>
       <c r="D506" t="n">
-        <v>109.46</v>
+        <v>109.21</v>
       </c>
       <c r="E506" t="n">
         <v>37.75</v>
@@ -11111,7 +11111,7 @@
         <v>3602872</v>
       </c>
       <c r="D507" t="n">
-        <v>109.64</v>
+        <v>109.46</v>
       </c>
       <c r="E507" t="n">
         <v>37.5</v>
@@ -11133,7 +11133,7 @@
         <v>3588642</v>
       </c>
       <c r="D508" t="n">
-        <v>109.67</v>
+        <v>109.64</v>
       </c>
       <c r="E508" t="n">
         <v>37.5625</v>
@@ -11155,7 +11155,7 @@
         <v>3546894</v>
       </c>
       <c r="D509" t="n">
-        <v>109.71</v>
+        <v>109.67</v>
       </c>
       <c r="E509" t="n">
         <v>37.625</v>
@@ -11177,7 +11177,7 @@
         <v>3547947</v>
       </c>
       <c r="D510" t="n">
-        <v>109.79</v>
+        <v>109.71</v>
       </c>
       <c r="E510" t="n">
         <v>37.5</v>
@@ -11199,7 +11199,7 @@
         <v>3659413</v>
       </c>
       <c r="D511" t="n">
-        <v>110.08</v>
+        <v>109.79</v>
       </c>
       <c r="E511" t="n">
         <v>37.625</v>
@@ -11221,7 +11221,7 @@
         <v>3609733</v>
       </c>
       <c r="D512" t="n">
-        <v>110.11</v>
+        <v>110.08</v>
       </c>
       <c r="E512" t="n">
         <v>37.625</v>
@@ -11243,7 +11243,7 @@
         <v>3620102</v>
       </c>
       <c r="D513" t="n">
-        <v>110.15</v>
+        <v>110.11</v>
       </c>
       <c r="E513" t="n">
         <v>37.5625</v>
@@ -11265,7 +11265,7 @@
         <v>3597892</v>
       </c>
       <c r="D514" t="n">
-        <v>110.5</v>
+        <v>110.15</v>
       </c>
       <c r="E514" t="n">
         <v>37.5625</v>
@@ -11287,7 +11287,7 @@
         <v>3643133</v>
       </c>
       <c r="D515" t="n">
-        <v>110.68</v>
+        <v>110.5</v>
       </c>
       <c r="E515" t="n">
         <v>37.75</v>
@@ -11309,7 +11309,7 @@
         <v>3631047</v>
       </c>
       <c r="D516" t="n">
-        <v>110.71</v>
+        <v>110.68</v>
       </c>
       <c r="E516" t="n">
         <v>37.625</v>
@@ -11335,7 +11335,7 @@
         <v>3880988</v>
       </c>
       <c r="D517" t="n">
-        <v>110.75</v>
+        <v>110.71</v>
       </c>
       <c r="E517" t="n">
         <v>37.5</v>
@@ -11357,7 +11357,7 @@
         <v>3857121</v>
       </c>
       <c r="D518" t="n">
-        <v>110.92</v>
+        <v>110.75</v>
       </c>
       <c r="E518" t="n">
         <v>37.5625</v>
@@ -11401,7 +11401,7 @@
         <v>3705419</v>
       </c>
       <c r="D520" t="n">
-        <v>111.37</v>
+        <v>110.92</v>
       </c>
       <c r="E520" t="n">
         <v>37.5625</v>
@@ -11423,7 +11423,7 @@
         <v>3631309</v>
       </c>
       <c r="D521" t="n">
-        <v>111.46</v>
+        <v>111.37</v>
       </c>
       <c r="E521" t="n">
         <v>37.375</v>
@@ -11445,7 +11445,7 @@
         <v>3750052</v>
       </c>
       <c r="D522" t="n">
-        <v>111.49</v>
+        <v>111.46</v>
       </c>
       <c r="E522" t="n">
         <v>37.4375</v>
@@ -11467,7 +11467,7 @@
         <v>3709414</v>
       </c>
       <c r="D523" t="n">
-        <v>111.52</v>
+        <v>111.49</v>
       </c>
       <c r="E523" t="n">
         <v>37.6875</v>
@@ -11489,7 +11489,7 @@
         <v>3745962</v>
       </c>
       <c r="D524" t="n">
-        <v>111.59</v>
+        <v>111.52</v>
       </c>
       <c r="E524" t="n">
         <v>37.5</v>
@@ -11511,7 +11511,7 @@
         <v>3784898</v>
       </c>
       <c r="D525" t="n">
-        <v>111.67</v>
+        <v>111.59</v>
       </c>
       <c r="E525" t="n">
         <v>37.5625</v>
@@ -11533,7 +11533,7 @@
         <v>3926458</v>
       </c>
       <c r="D526" t="n">
-        <v>112.01</v>
+        <v>111.67</v>
       </c>
       <c r="E526" t="n">
         <v>37.5</v>
@@ -11555,7 +11555,7 @@
         <v>3994573</v>
       </c>
       <c r="D527" t="n">
-        <v>112.17</v>
+        <v>112.01</v>
       </c>
       <c r="E527" t="n">
         <v>37.625</v>
@@ -11577,7 +11577,7 @@
         <v>3906529</v>
       </c>
       <c r="D528" t="n">
-        <v>112.21</v>
+        <v>112.17</v>
       </c>
       <c r="E528" t="n">
         <v>37.6875</v>
@@ -11599,7 +11599,7 @@
         <v>3821174</v>
       </c>
       <c r="D529" t="n">
-        <v>112.24</v>
+        <v>112.21</v>
       </c>
       <c r="E529" t="n">
         <v>37.625</v>
@@ -11621,7 +11621,7 @@
         <v>3729418</v>
       </c>
       <c r="D530" t="n">
-        <v>112.48</v>
+        <v>112.24</v>
       </c>
       <c r="E530" t="n">
         <v>39.9375</v>
@@ -11643,7 +11643,7 @@
         <v>3812115</v>
       </c>
       <c r="D531" t="n">
-        <v>112.71</v>
+        <v>112.48</v>
       </c>
       <c r="E531" t="n">
         <v>39.875</v>
@@ -11665,7 +11665,7 @@
         <v>3644962</v>
       </c>
       <c r="D532" t="n">
-        <v>112.8</v>
+        <v>112.71</v>
       </c>
       <c r="E532" t="n">
         <v>40.0625</v>
@@ -11687,7 +11687,7 @@
         <v>3592761</v>
       </c>
       <c r="D533" t="n">
-        <v>112.83</v>
+        <v>112.8</v>
       </c>
       <c r="E533" t="n">
         <v>40.0625</v>
@@ -11709,7 +11709,7 @@
         <v>3676507</v>
       </c>
       <c r="D534" t="n">
-        <v>112.89</v>
+        <v>112.83</v>
       </c>
       <c r="E534" t="n">
         <v>39.9375</v>
@@ -11731,7 +11731,7 @@
         <v>3672002</v>
       </c>
       <c r="D535" t="n">
-        <v>112.95</v>
+        <v>112.89</v>
       </c>
       <c r="E535" t="n">
         <v>39.9375</v>
@@ -27998,7 +27998,7 @@
       </c>
       <c r="F1273" t="inlineStr"/>
       <c r="G1273" t="n">
-        <v>44054294.14</v>
+        <v>44057000.14</v>
       </c>
       <c r="H1273" t="inlineStr"/>
     </row>
@@ -31196,7 +31196,7 @@
       </c>
       <c r="F1418" t="inlineStr"/>
       <c r="G1418" t="n">
-        <v>50598545.87</v>
+        <v>50628066.87</v>
       </c>
       <c r="H1418" t="inlineStr"/>
     </row>
@@ -31218,7 +31218,7 @@
       </c>
       <c r="F1419" t="inlineStr"/>
       <c r="G1419" t="n">
-        <v>51157559.993</v>
+        <v>51182478.993</v>
       </c>
       <c r="H1419" t="inlineStr"/>
     </row>
@@ -31750,7 +31750,7 @@
       </c>
       <c r="F1443" t="inlineStr"/>
       <c r="G1443" t="n">
-        <v>51564746.942</v>
+        <v>51569146.942</v>
       </c>
       <c r="H1443" t="inlineStr"/>
     </row>
@@ -32128,7 +32128,7 @@
       </c>
       <c r="F1460" t="inlineStr"/>
       <c r="G1460" t="n">
-        <v>53428777.364</v>
+        <v>53303363.364</v>
       </c>
       <c r="H1460" t="inlineStr"/>
     </row>
@@ -32364,7 +32364,7 @@
       </c>
       <c r="F1471" t="inlineStr"/>
       <c r="G1471" t="n">
-        <v>55081107.553</v>
+        <v>55084943.553</v>
       </c>
       <c r="H1471" t="inlineStr"/>
     </row>
@@ -32644,7 +32644,7 @@
       </c>
       <c r="F1484" t="inlineStr"/>
       <c r="G1484" t="n">
-        <v>61890800.993</v>
+        <v>61891566.993</v>
       </c>
       <c r="H1484" t="inlineStr"/>
     </row>
@@ -32688,7 +32688,7 @@
       </c>
       <c r="F1486" t="inlineStr"/>
       <c r="G1486" t="n">
-        <v>61722932.076</v>
+        <v>61717759.076</v>
       </c>
       <c r="H1486" t="inlineStr"/>
     </row>
@@ -32820,7 +32820,7 @@
       </c>
       <c r="F1492" t="inlineStr"/>
       <c r="G1492" t="n">
-        <v>57549505.399</v>
+        <v>57556557.399</v>
       </c>
       <c r="H1492" t="inlineStr"/>
     </row>
@@ -32842,7 +32842,7 @@
       </c>
       <c r="F1493" t="inlineStr"/>
       <c r="G1493" t="n">
-        <v>56278446.088</v>
+        <v>56231542.088</v>
       </c>
       <c r="H1493" t="inlineStr"/>
     </row>
@@ -33062,7 +33062,7 @@
       </c>
       <c r="F1503" t="inlineStr"/>
       <c r="G1503" t="n">
-        <v>60129333.818</v>
+        <v>60130226.818</v>
       </c>
       <c r="H1503" t="inlineStr"/>
     </row>
@@ -33100,7 +33100,7 @@
       </c>
       <c r="F1505" t="inlineStr"/>
       <c r="G1505" t="n">
-        <v>59046331.841</v>
+        <v>59046653.841</v>
       </c>
       <c r="H1505" t="inlineStr"/>
     </row>
@@ -33122,7 +33122,7 @@
       </c>
       <c r="F1506" t="inlineStr"/>
       <c r="G1506" t="n">
-        <v>58347586.213</v>
+        <v>58347731.213</v>
       </c>
       <c r="H1506" t="inlineStr"/>
     </row>
@@ -33144,7 +33144,7 @@
       </c>
       <c r="F1507" t="inlineStr"/>
       <c r="G1507" t="n">
-        <v>58584047.727</v>
+        <v>58584994.727</v>
       </c>
       <c r="H1507" t="inlineStr"/>
     </row>
@@ -33166,7 +33166,7 @@
       </c>
       <c r="F1508" t="inlineStr"/>
       <c r="G1508" t="n">
-        <v>59669950.587</v>
+        <v>59670177.587</v>
       </c>
       <c r="H1508" t="inlineStr"/>
     </row>
@@ -33188,7 +33188,7 @@
       </c>
       <c r="F1509" t="inlineStr"/>
       <c r="G1509" t="n">
-        <v>58024518.8</v>
+        <v>58024789.8</v>
       </c>
       <c r="H1509" t="inlineStr"/>
     </row>
@@ -33210,7 +33210,7 @@
       </c>
       <c r="F1510" t="inlineStr"/>
       <c r="G1510" t="n">
-        <v>57264087.786</v>
+        <v>57264548.786</v>
       </c>
       <c r="H1510" t="inlineStr"/>
     </row>
@@ -33232,7 +33232,7 @@
       </c>
       <c r="F1511" t="inlineStr"/>
       <c r="G1511" t="n">
-        <v>56145981.11</v>
+        <v>56146237.11</v>
       </c>
       <c r="H1511" t="inlineStr"/>
     </row>
@@ -33254,7 +33254,7 @@
       </c>
       <c r="F1512" t="inlineStr"/>
       <c r="G1512" t="n">
-        <v>56460309.744</v>
+        <v>56460373.744</v>
       </c>
       <c r="H1512" t="inlineStr"/>
     </row>
@@ -33276,7 +33276,7 @@
       </c>
       <c r="F1513" t="inlineStr"/>
       <c r="G1513" t="n">
-        <v>55872372.876</v>
+        <v>55872398.876</v>
       </c>
       <c r="H1513" t="inlineStr"/>
     </row>
@@ -33298,7 +33298,7 @@
       </c>
       <c r="F1514" t="inlineStr"/>
       <c r="G1514" t="n">
-        <v>55629131.143</v>
+        <v>55629217.143</v>
       </c>
       <c r="H1514" t="inlineStr"/>
     </row>
@@ -33320,7 +33320,7 @@
       </c>
       <c r="F1515" t="inlineStr"/>
       <c r="G1515" t="n">
-        <v>55628650.479</v>
+        <v>55628892.479</v>
       </c>
       <c r="H1515" t="inlineStr"/>
     </row>
@@ -33342,7 +33342,7 @@
       </c>
       <c r="F1516" t="inlineStr"/>
       <c r="G1516" t="n">
-        <v>55674183.733</v>
+        <v>55674505.733</v>
       </c>
       <c r="H1516" t="inlineStr"/>
     </row>
@@ -33364,7 +33364,7 @@
       </c>
       <c r="F1517" t="inlineStr"/>
       <c r="G1517" t="n">
-        <v>55246747.15</v>
+        <v>55246756.15</v>
       </c>
       <c r="H1517" t="inlineStr"/>
     </row>
@@ -33386,7 +33386,7 @@
       </c>
       <c r="F1518" t="inlineStr"/>
       <c r="G1518" t="n">
-        <v>55295684.162</v>
+        <v>55295794.162</v>
       </c>
       <c r="H1518" t="inlineStr"/>
     </row>
@@ -33408,7 +33408,7 @@
       </c>
       <c r="F1519" t="inlineStr"/>
       <c r="G1519" t="n">
-        <v>54752343.928</v>
+        <v>54752329.928</v>
       </c>
       <c r="H1519" t="inlineStr"/>
     </row>
@@ -33430,7 +33430,7 @@
       </c>
       <c r="F1520" t="inlineStr"/>
       <c r="G1520" t="n">
-        <v>55611791.663</v>
+        <v>55612023.663</v>
       </c>
       <c r="H1520" t="inlineStr"/>
     </row>
@@ -33452,7 +33452,7 @@
       </c>
       <c r="F1521" t="inlineStr"/>
       <c r="G1521" t="n">
-        <v>57362057.612</v>
+        <v>57362158.612</v>
       </c>
       <c r="H1521" t="inlineStr"/>
     </row>
@@ -33474,7 +33474,7 @@
       </c>
       <c r="F1522" t="inlineStr"/>
       <c r="G1522" t="n">
-        <v>60323415.161</v>
+        <v>60314877.836</v>
       </c>
       <c r="H1522" t="inlineStr"/>
     </row>
@@ -33710,7 +33710,7 @@
       </c>
       <c r="F1533" t="inlineStr"/>
       <c r="G1533" t="n">
-        <v>57182086.585</v>
+        <v>57181433.585</v>
       </c>
       <c r="H1533" t="inlineStr"/>
     </row>
@@ -33732,7 +33732,7 @@
       </c>
       <c r="F1534" t="inlineStr"/>
       <c r="G1534" t="n">
-        <v>55951832.971</v>
+        <v>55945733.807</v>
       </c>
       <c r="H1534" t="inlineStr"/>
     </row>
@@ -33754,7 +33754,7 @@
       </c>
       <c r="F1535" t="inlineStr"/>
       <c r="G1535" t="n">
-        <v>55098019.615</v>
+        <v>55098036.615</v>
       </c>
       <c r="H1535" t="inlineStr"/>
     </row>
@@ -33776,7 +33776,7 @@
       </c>
       <c r="F1536" t="inlineStr"/>
       <c r="G1536" t="n">
-        <v>54572458.523</v>
+        <v>54572824.523</v>
       </c>
       <c r="H1536" t="inlineStr"/>
     </row>
@@ -33820,7 +33820,7 @@
       </c>
       <c r="F1538" t="inlineStr"/>
       <c r="G1538" t="n">
-        <v>54931152.1</v>
+        <v>54914169.986</v>
       </c>
       <c r="H1538" t="inlineStr"/>
     </row>
@@ -33841,15 +33841,21 @@
         <v>25.375</v>
       </c>
       <c r="F1539" t="inlineStr"/>
-      <c r="G1539" t="inlineStr"/>
+      <c r="G1539" t="n">
+        <v>56070015.35</v>
+      </c>
       <c r="H1539" t="inlineStr"/>
     </row>
     <row r="1540">
       <c r="A1540" s="2" t="n">
         <v>46107</v>
       </c>
-      <c r="B1540" t="inlineStr"/>
-      <c r="C1540" t="inlineStr"/>
+      <c r="B1540" t="n">
+        <v>43534</v>
+      </c>
+      <c r="C1540" t="n">
+        <v>40433607</v>
+      </c>
       <c r="D1540" t="n">
         <v>1392.39</v>
       </c>
@@ -33869,10 +33875,26 @@
       <c r="D1541" t="n">
         <v>1404.43</v>
       </c>
-      <c r="E1541" t="inlineStr"/>
+      <c r="E1541" t="n">
+        <v>24.8125</v>
+      </c>
       <c r="F1541" t="inlineStr"/>
       <c r="G1541" t="inlineStr"/>
       <c r="H1541" t="inlineStr"/>
+    </row>
+    <row r="1542">
+      <c r="A1542" s="2" t="n">
+        <v>46111</v>
+      </c>
+      <c r="B1542" t="inlineStr"/>
+      <c r="C1542" t="inlineStr"/>
+      <c r="D1542" t="n">
+        <v>1419.32</v>
+      </c>
+      <c r="E1542" t="inlineStr"/>
+      <c r="F1542" t="inlineStr"/>
+      <c r="G1542" t="inlineStr"/>
+      <c r="H1542" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>